<commit_message>
Revise CraneSignal call sheet phone-first
</commit_message>
<xml_diff>
--- a/docs/call-sheets/cranesignal-maintenance-software-call-sheet-2026-09-21.xlsx
+++ b/docs/call-sheets/cranesignal-maintenance-software-call-sheet-2026-09-21.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Call Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phone Call Sheet" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Call Sheet'!$A$1:$N$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Phone Call Sheet'!$A$1:$I$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,23 +475,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="56" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -512,61 +507,36 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Fit</t>
+          <t>Best phone to try</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Public phone</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Public email</t>
+          <t>Why this number</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Backup email</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Source URL</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>What they sell</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>CraneSignal angle</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Recommended action</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Call status</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Last touch date</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="45" customHeight="1">
+          <t>Call note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -582,45 +552,36 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Very high</t>
+          <t>+1 347-909-1604</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>+1 347-909-1604; +1 201-241-3793</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Official/public company contact</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>sales@appworkco.com</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>https://appworkco.com/</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Multifamily maintenance software: work orders, technician tasks, inspections, make-ready boards, unit heat maps.</t>
-        </is>
-      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Free Texas maintenance-pain accounts for their sales team.</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Call first</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="45" customHeight="1">
+          <t>Best fit. Multifamily maintenance software. Call first with Texas maintenance-pain sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -636,45 +597,36 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Very high</t>
+          <t>877-995-3662 x513</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>877-995-3662 x513 sales; 877-995-3662 x500 general</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>Official sales line</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>sales@leonardo247.com</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>https://leonardo247.com/</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Multifamily property operations, maintenance, risk, due diligence, remote maintenance, turn workflows.</t>
-        </is>
-      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Maintenance pain + operational risk signals across Texas portfolios.</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Call first</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4" ht="45" customHeight="1">
+          <t>Best fit. Multifamily operations and maintenance platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -690,45 +642,36 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>888-222-0206 ext. 1</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>888-222-0206 ext. 1 sales</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>Official sales option</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>Info@MaintenanceCare.com</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>https://www.maintenancecare.com/work-order-software-for-apartment-maintenance</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>CMMS/work-order software for apartment maintenance and facilities.</t>
-        </is>
-      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Texas apartments with visible repair, response-time, and preventive-maintenance pain.</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Call first</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="45" customHeight="1">
+          <t>Strong apartment maintenance/work-order fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -744,45 +687,36 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>+1 530-746-8178</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>+1 530-746-8178</t>
+          <t>Medium-high</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
+          <t>Public app/developer support listing</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
           <t>support@zinspector.com</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>https://zinspector.com/</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Property inspection software, tenant self-inspections, AI inspection reports, work-order-connected workflows.</t>
-        </is>
-      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Properties with move-in, inspection, condition, or maintenance complaint signals.</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Call first</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6" ht="45" customHeight="1">
+          <t>Inspection and maintenance workflow fit. Good for move-in, condition, and repair signals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -798,41 +732,32 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>206-900-9466</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>206-900-9466</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Official help/contact phone</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>https://latchel.com/</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>AI front office and maintenance engine: maintenance calls, troubleshooting, dispatch, visibility.</t>
-        </is>
-      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Properties with after-hours, unresolved maintenance, and resident-complaint signals.</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Call first</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="45" customHeight="1">
+          <t>Strong maintenance coordination fit. Good for after-hours and unresolved maintenance pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -848,41 +773,32 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>913-513-4480</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>913-513-4480</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Official company phone</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>https://lula.life/</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Maintenance coordination, vendor network, after-hours maintenance, make-ready service, AI scheduling.</t>
-        </is>
-      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Properties where owners/operators likely need maintenance capacity or vendor help.</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Call first</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8" ht="45" customHeight="1">
+          <t>Strong maintenance coordination and vendor network fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -898,45 +814,36 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>+1 619-752-4422</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>+1 (619) 752-4422</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
+          <t>Official company phone</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
           <t>support@taskestate.com</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>https://taskestate.com/</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Property maintenance and work-order management for resident requests, approvals, inspections, vendors, assets.</t>
-        </is>
-      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Texas operators with messy resident maintenance workflows.</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Call first</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="45" customHeight="1">
+          <t>Smaller vendor with clear work-order and maintenance fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
@@ -952,37 +859,36 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
+          <t>+1 647-797-1997</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Official contact phone</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>https://www.suitespot.ai/</t>
+          <t>info@suitespot.ai</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>AI-powered multifamily maintenance and capital operations software.</t>
+          <t>https://www.suitespot.ai/integrations</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Texas properties with workload, work-order, or capital-opportunity signals.</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Find named sales/BD</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10" ht="45" customHeight="1">
+          <t>Strong AI multifamily maintenance and capital operations fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
@@ -998,37 +904,36 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
+          <t>+1 605-646-4102</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Medium-high</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Google Play developer listing</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
+          <t>support@propertymeld.com</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
           <t>https://propertymeld.com/</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Property maintenance automation.</t>
-        </is>
-      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Texas properties with public maintenance complaints and slow-resolution signals.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Find named sales/BD</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="45" customHeight="1">
+          <t>Very strong fit. Note: help center says no phone support, so this may route poorly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
@@ -1044,37 +949,36 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
+          <t>+1 617-877-8802</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Low-medium</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Third-party company listing</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://vendoroo.ai/</t>
+          <t>info@mezo.io</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>AI maintenance intake and automation for property operations.</t>
+          <t>https://www.mezo.io/</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Texas operators with support-ticket and intake pain.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Find named sales/BD</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12" ht="45" customHeight="1">
+          <t>Strong AI maintenance intake fit. If this fails, use Property Meld route because Mezo was acquired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
       <c r="A12" s="3" t="n">
         <v>11</v>
       </c>
@@ -1090,41 +994,32 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Medium-high</t>
+          <t>(877) 501-7117</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>(877) 501-7117; +1 (212) 501-7117</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr">
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Official US/Canada phone</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>https://www.buildinglink.io/</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Building/community operations software with maintenance requests, preventive tasks, vendors, assets, packages, communications.</t>
-        </is>
-      </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Higher-end multifamily/condo communities with operations pain.</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr"/>
-      <c r="N12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13" ht="45" customHeight="1">
+          <t>Good building operations and maintenance request fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
       <c r="A13" s="3" t="n">
         <v>12</v>
       </c>
@@ -1140,45 +1035,36 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Medium-high</t>
+          <t>(844) 800-7109</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>(844) 800-7109 support</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
+          <t>Public support/general line</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
           <t>info@vts.com; support@vts.com</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>https://www.vts.com/vts-activate-multifamily</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Resident experience and building operations: work orders, maintenance, access, communications, packages, payments.</t>
-        </is>
-      </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Maintenance plus resident-experience pain accounts.</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr"/>
-      <c r="N13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="45" customHeight="1">
+          <t>Good product fit, bigger company.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
       <c r="A14" s="3" t="n">
         <v>13</v>
       </c>
@@ -1194,37 +1080,36 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
+          <t>+1 773-673-9223</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
           <t>Medium-high</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Google Play developer listing</t>
+        </is>
+      </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
+          <t>support@livly.io</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
           <t>https://www.livly.io/</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Multifamily resident app and property hub with payments, maintenance requests, move-in checklists, resident events, packages, access.</t>
-        </is>
-      </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Resident app plus maintenance-friction accounts.</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>Find named sales/BD</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
-      <c r="N14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15" ht="45" customHeight="1">
+          <t>Resident app with maintenance requests. Good but not maintenance-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
       <c r="A15" s="3" t="n">
         <v>14</v>
       </c>
@@ -1240,37 +1125,32 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Medium-high</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr">
+          <t>1-866-729-5327</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Official support phone</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>https://www.gozego.com/</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Multifamily workflow automation: payments, utilities, resident app, move-in/move-out, maintenance requests.</t>
-        </is>
-      </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Resident workflow and maintenance-request accounts.</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>Find named sales/BD</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
-      <c r="N15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16" ht="45" customHeight="1">
+          <t>Resident workflow and maintenance request fit. Bigger platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1">
       <c r="A16" s="3" t="n">
         <v>15</v>
       </c>
@@ -1286,37 +1166,36 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="3" t="inlineStr"/>
+          <t>1 (888) 883-8046</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Official phone</t>
+        </is>
+      </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>https://www.snapinspect.com/property-maintenance-software</t>
+          <t>contact@snapinspect.com</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Property inspection app/software, remote inspections, maintenance workflows, reports, photo documentation.</t>
+          <t>https://www.snapinspect.com/</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Inspection, move-in/move-out, and unit-condition accounts.</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr"/>
-      <c r="L16" s="3" t="inlineStr"/>
-      <c r="M16" s="3" t="inlineStr"/>
-      <c r="N16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17" ht="45" customHeight="1">
+          <t>Good inspection and property maintenance fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="44" customHeight="1">
       <c r="A17" s="3" t="n">
         <v>16</v>
       </c>
@@ -1332,41 +1211,32 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>+1 800 321 8770</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+1 800 321 8770</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr"/>
-      <c r="G17" s="3" t="inlineStr">
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Official company phone</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>https://www.mrisoftware.com/solutions/building-maintenance-software/facilities-work-order-system/</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Building operations and property management work-order software.</t>
-        </is>
-      </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Enterprise facilities/work-order opportunities.</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
-      <c r="N17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="45" customHeight="1">
+          <t>Enterprise building maintenance/work-order fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="44" customHeight="1">
       <c r="A18" s="3" t="n">
         <v>17</v>
       </c>
@@ -1382,41 +1252,32 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Medium-high</t>
+          <t>+1-888-607-3667</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>+1-888-607-3667; +1-786-373-5842</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr">
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Official toll-free phone</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>https://www.doorloop.com/contact</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Property management software with maintenance, AI maintenance handling, work orders, vendor payments, accounting, leasing.</t>
-        </is>
-      </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Broad PMS buyer; pitch as lead-data partnership, not replacement software.</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr"/>
-      <c r="L18" s="3" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr"/>
-      <c r="N18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19" ht="45" customHeight="1">
+          <t>Broad PMS with maintenance. Good second wave.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="44" customHeight="1">
       <c r="A19" s="3" t="n">
         <v>18</v>
       </c>
@@ -1432,41 +1293,32 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>877-396-7876</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>877-396-7876 sales; (617) 829-9570 corporate</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr"/>
-      <c r="G19" s="3" t="inlineStr">
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Official sales phone</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>https://www.buildium.com/contact-us/</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Property management software with maintenance requests, resident center, and maintenance contact center.</t>
-        </is>
-      </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Broad PMS/RealPage-owned; useful market context but not first call.</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr"/>
-      <c r="L19" s="3" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr"/>
-      <c r="N19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="45" customHeight="1">
+          <t>Broad PMS with maintenance. RealPage-owned, so second wave.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
       <c r="A20" s="3" t="n">
         <v>19</v>
       </c>
@@ -1482,41 +1334,32 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>(888) 702-0971</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>(888) 702-0971</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr"/>
-      <c r="G20" s="3" t="inlineStr">
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Official phone</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>https://www.myresman.com/contact-us/</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Multifamily property management software with maintenance, resident portal, contact center, AI resident assistant.</t>
-        </is>
-      </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Texas-linked broad PMS; pitch cautiously.</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr"/>
-      <c r="L20" s="3" t="inlineStr"/>
-      <c r="M20" s="3" t="inlineStr"/>
-      <c r="N20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21" ht="45" customHeight="1">
+          <t>Broad multifamily PMS. Texas-linked, but not first wave.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1">
       <c r="A21" s="3" t="n">
         <v>20</v>
       </c>
@@ -1532,41 +1375,32 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>866.648.1536</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>866.648.1536</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr">
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Official phone</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>https://www.appfolio.com/</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Property management platform with maintenance, resident service, communications, and AI operations.</t>
-        </is>
-      </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Large PMS; call only after proving sample value.</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr"/>
-      <c r="L21" s="3" t="inlineStr"/>
-      <c r="M21" s="3" t="inlineStr"/>
-      <c r="N21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="45" customHeight="1">
+          <t>Large PMS. Call after the sample proves value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
       <c r="A22" s="3" t="n">
         <v>21</v>
       </c>
@@ -1582,41 +1416,32 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>(800) 866-1144</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>(800) 866-1144</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr"/>
-      <c r="G22" s="3" t="inlineStr">
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Official phone</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>https://www.yardibreeze.com/contact-us/</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Property management software for residential, commercial, affordable, self storage, HOA/condo, manufactured housing.</t>
-        </is>
-      </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Large platform; hard first target.</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr"/>
-      <c r="L22" s="3" t="inlineStr"/>
-      <c r="M22" s="3" t="inlineStr"/>
-      <c r="N22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23" ht="45" customHeight="1">
+          <t>Large PMS. Harder first target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="44" customHeight="1">
       <c r="A23" s="3" t="n">
         <v>22</v>
       </c>
@@ -1632,45 +1457,36 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Medium-high</t>
+          <t>1.800.700.2097</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>1.800.700.2097</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
+          <t>Official phone</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
           <t>sales@entrata.com</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>https://www.entrata.com/products/facility-management</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Facilities app for maintenance staff to view, edit, complete work orders and inspections.</t>
-        </is>
-      </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Strong fit but large company; better with named BD contact.</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr"/>
-      <c r="M23" s="3" t="inlineStr"/>
-      <c r="N23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="45" customHeight="1">
+          <t>Strong facilities product fit, large company.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1">
       <c r="A24" s="3" t="n">
         <v>23</v>
       </c>
@@ -1686,45 +1502,36 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Medium-high</t>
+          <t>1 (833) 767-8736</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>1 (833) 767-8736</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
+          <t>Official company phone</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
           <t>help@sightplan.com</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>https://smartrent.com/</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Smart apartment and operations tools; SightPlan historically covered resident service, tasks, work orders, inspections.</t>
-        </is>
-      </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Smart operations and maintenance pain accounts.</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr"/>
-      <c r="L24" s="3" t="inlineStr"/>
-      <c r="M24" s="3" t="inlineStr"/>
-      <c r="N24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25" ht="45" customHeight="1">
+          <t>Good smart operations and maintenance fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1">
       <c r="A25" s="4" t="n">
         <v>24</v>
       </c>
@@ -1740,37 +1547,36 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="4" t="inlineStr"/>
+          <t>+91 98848 02586</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Low-medium</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Public company/social listing</t>
+        </is>
+      </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
+          <t>getsmart@facilio.com</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
           <t>https://facilio.com/</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>Connected CMMS and property operations platform for work orders, costs, SLAs, tenant satisfaction, vendors, portfolio analytics.</t>
-        </is>
-      </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Enterprise property operations, more commercial than apartment-only.</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>Research later</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr"/>
-      <c r="L25" s="4" t="inlineStr"/>
-      <c r="M25" s="4" t="inlineStr"/>
-      <c r="N25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26" ht="45" customHeight="1">
+          <t>Enterprise FM platform, not apartment-specific. Low priority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="44" customHeight="1">
       <c r="A26" s="4" t="n">
         <v>25</v>
       </c>
@@ -1786,45 +1592,36 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>+1 (844) 664-4400</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>+1 (844) 664-4400</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
+          <t>Official help-center phone</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
           <t>support@gofmx.com</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>https://help.gofmx.com/hc/en-us</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>Facilities and maintenance management software: work orders, preventive maintenance, reporting, scheduling, inventory.</t>
-        </is>
-      </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
           <t>Facilities fit, but less apartment-specific.</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>Research later</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr"/>
-      <c r="L26" s="4" t="inlineStr"/>
-      <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27" ht="45" customHeight="1">
+    </row>
+    <row r="27" ht="44" customHeight="1">
       <c r="A27" s="4" t="n">
         <v>26</v>
       </c>
@@ -1840,37 +1637,36 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Low-medium</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="inlineStr"/>
+          <t>+1 (775) 210-5128</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Official help-center phone</t>
+        </is>
+      </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
+          <t>mail@limblecmms.com</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
           <t>https://limblecmms.com/</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>CMMS for work orders, preventive maintenance, assets, QR codes, technician workflows.</t>
-        </is>
-      </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Broad CMMS, not apartment-specific enough for first sprint.</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>Research later</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr"/>
-      <c r="L27" s="4" t="inlineStr"/>
-      <c r="M27" s="4" t="inlineStr"/>
-      <c r="N27" s="4" t="inlineStr"/>
-    </row>
-    <row r="28" ht="45" customHeight="1">
+          <t>Broad CMMS. Lower priority for apartment-specific calling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="44" customHeight="1">
       <c r="A28" s="4" t="n">
         <v>27</v>
       </c>
@@ -1886,37 +1682,36 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Low-medium</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr"/>
-      <c r="F28" s="4" t="inlineStr"/>
+          <t>+1 (323) 880-0280</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Official help/app support phone</t>
+        </is>
+      </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
+          <t>info@onupkeep.com</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
           <t>https://upkeep.com/</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>CMMS/work-order platform with multifamily/property-management use cases.</t>
-        </is>
-      </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Broad CMMS; use only after apartment-specific vendors.</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>Research later</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr"/>
-      <c r="L28" s="4" t="inlineStr"/>
-      <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29" ht="45" customHeight="1">
+          <t>Broad CMMS. Good category, lower apartment specificity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="1">
       <c r="A29" s="4" t="n">
         <v>28</v>
       </c>
@@ -1932,37 +1727,36 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Low-medium</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="4" t="inlineStr"/>
+          <t>415-548-4001</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Official terms/company phone</t>
+        </is>
+      </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
+          <t>info@getmaintainx.com</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
           <t>https://www.getmaintainx.com/</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>Maintenance operations/work-order software.</t>
-        </is>
-      </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Strong maintenance category but broader manufacturing/facilities positioning.</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>Research later</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr"/>
-      <c r="L29" s="4" t="inlineStr"/>
-      <c r="M29" s="4" t="inlineStr"/>
-      <c r="N29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30" ht="45" customHeight="1">
+          <t>Broad CMMS. Property-management use case exists, but not first wave.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="44" customHeight="1">
       <c r="A30" s="4" t="n">
         <v>29</v>
       </c>
@@ -1978,41 +1772,36 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Medium-high</t>
+          <t>1-888-666-1855</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>1-888-666-1855 support</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Public app/support phone</t>
+        </is>
+      </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
+          <t>support@happy.co</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
           <t>https://happy.co/</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>Property management and maintenance software with AI-powered maintenance automation and work orders.</t>
-        </is>
-      </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Good fit; use once free sample exists.</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K30" s="4" t="inlineStr"/>
-      <c r="L30" s="4" t="inlineStr"/>
-      <c r="M30" s="4" t="inlineStr"/>
-      <c r="N30" s="4" t="inlineStr"/>
-    </row>
-    <row r="31" ht="45" customHeight="1">
+          <t>Good maintenance automation fit. Support phone may not route to sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="1">
       <c r="A31" s="4" t="n">
         <v>30</v>
       </c>
@@ -2028,49 +1817,35 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Medium-high</t>
+          <t>(888) 333-4617</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>(888) 333-4617</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr">
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Official phone</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>https://eworkorders.com/property-management-maintenance-management-software-cmms/</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>Property maintenance CMMS for work orders, assets, vendors, inspections, compliance, dashboards.</t>
-        </is>
-      </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Good property maintenance fit; not fully multifamily-specific.</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>Second wave</t>
-        </is>
-      </c>
-      <c r="K31" s="4" t="inlineStr"/>
-      <c r="L31" s="4" t="inlineStr"/>
-      <c r="M31" s="4" t="inlineStr"/>
-      <c r="N31" s="4" t="inlineStr"/>
+          <t>Good property maintenance CMMS fit, not fully multifamily-specific.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N31"/>
-  <dataValidations count="1">
-    <dataValidation sqref="K2:K31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Not started,Called - no answer,Left voicemail,Connected,Send sample,Not fit,Do not call"</formula1>
-    </dataValidation>
-  </dataValidations>
+  <autoFilter ref="A1:I31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2080,14 +1855,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="112" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Goal</t>
@@ -2095,127 +1870,67 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Call apartment maintenance/facilities software vendors and test whether CraneSignal lead intelligence is valuable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1">
+          <t>Call the best public phone number for each vendor and ask who should receive CraneSignal free Texas maintenance-pain sample leads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Primary offer</t>
+          <t>Best opener</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>We pulled Texas apartment communities with visible maintenance pain signals and can share a few free accounts your sales team should look at.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="36" customHeight="1">
+          <t>Hi, this is Drew with CraneSignal. We are mapping Texas apartment communities showing public maintenance pain signals. I pulled a few accounts your sales team may want. Who is the best person to send that to?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Best first outcome</t>
+          <t>What changed</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>They ask to see the sample lead pack or tell us who on the sales/BD team should review it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
+          <t>Removed the call-notes PDF template and removed vague named-person instructions. The sheet now gives a best phone number for every company.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
+          <t>Number confidence</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>High means official site/help/contact/terms. Medium means public app listing or support line. Low means third-party public listing and should be checked before repeated calls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>First wave</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Call Tier A first. If a number routes to support, ask for sales, partnerships, business development, or revenue leadership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
           <t>Do not say</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Do not say every apartment needs software. Say we find timely accounts with evidence-backed maintenance pain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Editable columns</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Call status, Owner, Last touch date, Notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Example status values</t>
-        </is>
-      </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Not started, Called - no answer, Left voicemail, Connected, Send sample, Not fit, Do not call.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>First wave</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Call Tier A first: AppWork, Leonardo247, Maintenance Care, zInspector, Latchel, Lula, TaskEstate, SuiteSpot, Property Meld, Mezo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Call opener</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Hi, this is Drew with CraneSignal. We are mapping Texas apartment communities showing public maintenance pain signals. I pulled a few accounts your sales team may want. Who is the best person to send that to?</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Voicemail</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Hi, this is Drew with CraneSignal. I found a few Texas apartment accounts that look relevant for your maintenance sales team because residents are publicly complaining about repairs and response times. I can send the free sample if useful.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Email follow-up</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Subject: Free Texas apartment maintenance-pain accounts. Body: I pulled a small sample of Texas apartment communities with public maintenance pain signals and thought your sales team may want to review them. Worth sending over?</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Assumption</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Phone numbers and emails are public-source contacts from the ICP research pass; verify before high-volume dialing.</t>
+          <t>Do not say every apartment needs software. Say we found timely accounts with evidence-backed maintenance pain.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add caller context to CraneSignal call sheet
</commit_message>
<xml_diff>
--- a/docs/call-sheets/cranesignal-maintenance-software-call-sheet-2026-09-21.xlsx
+++ b/docs/call-sheets/cranesignal-maintenance-software-call-sheet-2026-09-21.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Phone Call Sheet'!$A$1:$I$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Phone Call Sheet'!$A$1:$J$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,12 +20,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -37,6 +44,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="6">
@@ -90,29 +103,40 @@
       </bottom>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -475,18 +499,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="56" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -507,36 +532,41 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Best phone to try</t>
+          <t>Website</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Best phone</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Why this number</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Backup email</t>
+          <t>Ask for</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Source URL</t>
+          <t>Why they might care</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Call note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="44" customHeight="1">
+          <t>First question</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Fallback / note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -550,38 +580,43 @@
           <t>AppWork</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>https://appworkco.com/</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>+1 347-909-1604</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Official/public company contact</t>
-        </is>
-      </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>sales@appworkco.com</t>
+          <t>Sales / founder / revenue leader</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://appworkco.com/</t>
+          <t>They sell exactly into multifamily maintenance teams.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Best fit. Multifamily maintenance software. Call first with Texas maintenance-pain sample.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44" customHeight="1">
+          <t>Do you sell into Texas multifamily operators today?</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>If routed to support, ask for sales or partnerships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -595,38 +630,43 @@
           <t>Leonardo247</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>https://leonardo247.com/</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>877-995-3662 x513</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Official sales line</t>
-        </is>
-      </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>sales@leonardo247.com</t>
+          <t>Sales / enterprise sales / partnerships</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://leonardo247.com/</t>
+          <t>They sell property operations and maintenance software to multifamily.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Best fit. Multifamily operations and maintenance platform.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44" customHeight="1">
+          <t>Would a sourced list of Texas properties with maintenance-risk signals help your sales team?</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Use sales extension first; general extension is x500.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -640,38 +680,43 @@
           <t>Maintenance Care</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.maintenancecare.com/work-order-software-for-apartment-maintenance</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>888-222-0206 ext. 1</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Official sales option</t>
-        </is>
-      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Info@MaintenanceCare.com</t>
+          <t>Sales / account executive</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.maintenancecare.com/work-order-software-for-apartment-maintenance</t>
+          <t>Clear apartment maintenance/work-order buyer.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Strong apartment maintenance/work-order fit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44" customHeight="1">
+          <t>Do you have reps prospecting apartment operators in Texas?</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Use sales option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -685,38 +730,43 @@
           <t>zInspector</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://zinspector.com/</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>+1 530-746-8178</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Medium-high</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Public app/developer support listing</t>
-        </is>
-      </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>support@zinspector.com</t>
+          <t>Sales / partnerships</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://zinspector.com/</t>
+          <t>Inspection and condition data maps well to move-in and repair pain.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Inspection and maintenance workflow fit. Good for move-in, condition, and repair signals.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44" customHeight="1">
+          <t>Would properties with inspection or move-in condition complaints be useful leads?</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>If support answers, ask who handles new business.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -730,34 +780,43 @@
           <t>Latchel</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>https://latchel.com/</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>206-900-9466</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Official help/contact phone</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Sales / growth / partnerships</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://latchel.com/</t>
+          <t>They handle maintenance coordination, calls, troubleshooting, dispatch.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Strong maintenance coordination fit. Good for after-hours and unresolved maintenance pain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="44" customHeight="1">
+          <t>Do you want Texas operators showing public unresolved-maintenance pain?</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Ask for the team handling property manager growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -771,34 +830,43 @@
           <t>Lula</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>https://lula.life/</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>913-513-4480</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Official company phone</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Sales / partnerships</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://lula.life/</t>
+          <t>Maintenance coordination and vendor network fits urgent maintenance pain.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Strong maintenance coordination and vendor network fit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="44" customHeight="1">
+          <t>Would a list of Texas operators with visible maintenance backlog signals help?</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Ask for property management sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -812,38 +880,43 @@
           <t>TaskEstate</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>https://taskestate.com/</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>+1 619-752-4422</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Official company phone</t>
-        </is>
-      </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>support@taskestate.com</t>
+          <t>Founder / sales / partnerships</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://taskestate.com/</t>
+          <t>Smaller vendor, clear maintenance workflow fit.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Smaller vendor with clear work-order and maintenance fit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="44" customHeight="1">
+          <t>Are you looking for more apartment maintenance software leads in Texas?</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Small company: ask directly for the owner of sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
@@ -857,38 +930,43 @@
           <t>SuiteSpot</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.suitespot.ai/</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>+1 647-797-1997</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Official contact phone</t>
-        </is>
-      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>info@suitespot.ai</t>
+          <t>Sales / partnerships / revenue leader</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://www.suitespot.ai/integrations</t>
+          <t>AI multifamily maintenance and capital operations fit.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Strong AI multifamily maintenance and capital operations fit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="44" customHeight="1">
+          <t>Would maintenance-pain evidence help you prioritize Texas accounts?</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>If no sales route, use info@suitespot.ai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
@@ -902,38 +980,43 @@
           <t>Property Meld</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>https://propertymeld.com/</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>+1 605-646-4102</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Medium-high</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Google Play developer listing</t>
-        </is>
-      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>support@propertymeld.com</t>
+          <t>Sales / partnerships</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://propertymeld.com/</t>
+          <t>Very strong maintenance automation fit.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Very strong fit. Note: help center says no phone support, so this may route poorly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="44" customHeight="1">
+          <t>Do you want a few Texas properties where residents publicly complain about repairs?</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Phone may route poorly; backup email support@propertymeld.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
@@ -947,903 +1030,1076 @@
           <t>Mezo</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mezo.io/</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>+1 617-877-8802</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Low-medium</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Third-party company listing</t>
-        </is>
-      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>info@mezo.io</t>
+          <t>Founder / sales / Property Meld contact</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://www.mezo.io/</t>
+          <t>AI maintenance intake fit, but company/contact trail is weaker.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Strong AI maintenance intake fit. If this fails, use Property Meld route because Mezo was acquired.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="44" customHeight="1">
-      <c r="A12" s="3" t="n">
+          <t>Who is the right person for AI maintenance sales lead data?</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>If number fails, route through Property Meld because Mezo was acquired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>BuildingLink</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.buildinglink.io/</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>(877) 501-7117</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Official US/Canada phone</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.buildinglink.io/</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>Good building operations and maintenance request fit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="44" customHeight="1">
-      <c r="A13" s="3" t="n">
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Sales / multifamily sales</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Building operations and maintenance requests.</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Do you sell into apartment communities where resident operations are visibly strained?</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>US/Canada line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>VTS Activate Multifamily</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vts.com/vts-activate-multifamily</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>(844) 800-7109</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Public support/general line</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>info@vts.com; support@vts.com</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>https://www.vts.com/vts-activate-multifamily</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Good product fit, bigger company.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="44" customHeight="1">
-      <c r="A14" s="3" t="n">
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Sales / multifamily team</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Resident experience plus building operations.</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Would maintenance plus resident-experience pain signals help your team?</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Support/general line; ask for Activate Multifamily sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Livly</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.livly.io/</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>+1 773-673-9223</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Medium-high</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Google Play developer listing</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>support@livly.io</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>https://www.livly.io/</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Resident app with maintenance requests. Good but not maintenance-only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="44" customHeight="1">
-      <c r="A15" s="3" t="n">
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Sales / partnerships</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Resident app with maintenance requests.</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Do you prospect apartment communities with resident experience issues?</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Backup support@livly.io.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Zego</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gozego.com/</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>1-866-729-5327</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Official support phone</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>https://www.gozego.com/</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>Resident workflow and maintenance request fit. Bigger platform.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="44" customHeight="1">
-      <c r="A16" s="3" t="n">
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Sales / resident experience sales</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Resident workflow and maintenance request system.</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Do Texas resident-workflow pain signals help your prospecting?</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Official support line; ask for sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>SnapInspect</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.snapinspect.com/</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>1 (888) 883-8046</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Official phone</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>contact@snapinspect.com</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>https://www.snapinspect.com/</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Good inspection and property maintenance fit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="44" customHeight="1">
-      <c r="A17" s="3" t="n">
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Sales / partnerships</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Inspection and property maintenance workflows.</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Would inspection/move-in condition complaint leads be useful?</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Backup contact@snapinspect.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>MRI Software / MRI Angus</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.mrisoftware.com/solutions/building-maintenance-software/facilities-work-order-system/</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>+1 800 321 8770</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Official company phone</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mrisoftware.com/solutions/building-maintenance-software/facilities-work-order-system/</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Enterprise building maintenance/work-order fit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="44" customHeight="1">
-      <c r="A18" s="3" t="n">
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>MRI Angus sales / building maintenance sales</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise building maintenance and work-order system.</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Who handles lead data or partnerships for MRI Angus?</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Large company: expect routing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="A18" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>DoorLoop</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.doorloop.com/contact</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>+1-888-607-3667</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Official toll-free phone</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>https://www.doorloop.com/contact</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Broad PMS with maintenance. Good second wave.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="44" customHeight="1">
-      <c r="A19" s="3" t="n">
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Sales / partnerships</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Broad PMS with AI maintenance/work orders.</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Do you want Texas apartment operators with public maintenance complaints?</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Backup USA number +1-786-373-5842.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Buildium</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>https://www.buildium.com/contact-us/</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>877-396-7876</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Official sales phone</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.buildium.com/contact-us/</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>Broad PMS with maintenance. RealPage-owned, so second wave.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="44" customHeight="1">
-      <c r="A20" s="3" t="n">
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Sales / partnerships</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>PMS with maintenance requests and contact center.</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Who reviews prospecting data partnerships for Buildium sales?</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>RealPage-owned, second wave.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>ResMan</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.myresman.com/contact-us/</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>(888) 702-0971</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Official phone</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>https://www.myresman.com/contact-us/</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Broad multifamily PMS. Texas-linked, but not first wave.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="44" customHeight="1">
-      <c r="A21" s="3" t="n">
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Sales / partnerships</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Multifamily PMS with maintenance and resident portal.</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>Would Texas operational-pain account lists help ResMan reps?</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Texas-linked broad PMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="50" customHeight="1">
+      <c r="A21" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>AppFolio</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>https://www.appfolio.com/</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>866.648.1536</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Official phone</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.appfolio.com/</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Large PMS. Call after the sample proves value.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="44" customHeight="1">
-      <c r="A22" s="3" t="n">
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Sales / partnerships</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Large PMS with maintenance and resident service.</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Who handles sales intelligence or lead partnerships?</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Large company; use after sample is strong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="50" customHeight="1">
+      <c r="A22" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Yardi Breeze</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.yardibreeze.com/contact-us/</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>(800) 866-1144</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Official phone</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yardibreeze.com/contact-us/</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>Large PMS. Harder first target.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="44" customHeight="1">
-      <c r="A23" s="3" t="n">
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Sales / partnerships</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Large PMS serving residential portfolios.</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Who reviews new account intelligence for Yardi Breeze sales?</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Large company; likely hard to route.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="50" customHeight="1">
+      <c r="A23" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Entrata Facilities</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>https://www.entrata.com/products/facility-management</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>1.800.700.2097</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Official phone</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>sales@entrata.com</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>https://www.entrata.com/products/facility-management</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>Strong facilities product fit, large company.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="44" customHeight="1">
-      <c r="A24" s="3" t="n">
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Facilities product sales / partnerships</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Facilities app for maintenance work orders and inspections.</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Would Texas properties with visible maintenance complaints be useful?</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Backup sales@entrata.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="50" customHeight="1">
+      <c r="A24" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>SmartRent / SightPlan</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>https://smartrent.com/</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>1 (833) 767-8736</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Official company phone</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>help@sightplan.com</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>https://smartrent.com/</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Good smart operations and maintenance fit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="44" customHeight="1">
-      <c r="A25" s="4" t="n">
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Sales / SightPlan or operations sales</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Smart operations, resident service, tasks, inspections.</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Who handles sales data for property operations products?</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Backup help@sightplan.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="50" customHeight="1">
+      <c r="A25" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Facilio</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>https://facilio.com/</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>+91 98848 02586</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Low-medium</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Public company/social listing</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>getsmart@facilio.com</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>https://facilio.com/</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>Enterprise FM platform, not apartment-specific. Low priority.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="44" customHeight="1">
-      <c r="A26" s="4" t="n">
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Sales / partnerships</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Enterprise property operations; less apartment-specific.</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>Do you sell into US multifamily, or mostly commercial facilities?</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>Low priority unless they confirm multifamily.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="50" customHeight="1">
+      <c r="A26" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>FMX</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>https://www.gofmx.com/</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>+1 (844) 664-4400</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>Official help-center phone</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>support@gofmx.com</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>https://help.gofmx.com/hc/en-us</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>Facilities fit, but less apartment-specific.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="44" customHeight="1">
-      <c r="A27" s="4" t="n">
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Sales / property management vertical</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Facilities and maintenance management.</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>Do you actively target apartment or property management companies?</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>Less apartment-specific.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="50" customHeight="1">
+      <c r="A27" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Limble CMMS</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>https://limblecmms.com/</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>+1 (775) 210-5128</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Official help-center phone</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>mail@limblecmms.com</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>https://limblecmms.com/</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>Broad CMMS. Lower priority for apartment-specific calling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="44" customHeight="1">
-      <c r="A28" s="4" t="n">
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Sales / property management use case</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Broad CMMS, lower apartment specificity.</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>Do you have a multifamily/property management vertical?</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>Only pursue if they say yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="50" customHeight="1">
+      <c r="A28" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>UpKeep</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>https://upkeep.com/</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>+1 (323) 880-0280</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Official help/app support phone</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>info@onupkeep.com</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>https://upkeep.com/</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>Broad CMMS. Good category, lower apartment specificity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="44" customHeight="1">
-      <c r="A29" s="4" t="n">
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Sales / property management use case</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Broad CMMS with property management use case.</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>Do you have a team selling into multifamily or apartment operators?</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>Lower priority than apartment-native vendors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="50" customHeight="1">
+      <c r="A29" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>MaintainX</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>https://www.getmaintainx.com/</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>415-548-4001</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Official terms/company phone</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>info@getmaintainx.com</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>https://www.getmaintainx.com/</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>Broad CMMS. Property-management use case exists, but not first wave.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="44" customHeight="1">
-      <c r="A30" s="4" t="n">
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Sales / property management use case</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>Broad maintenance ops software.</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>Do you sell into apartment maintenance teams or mostly industrial?</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>Lower priority unless they confirm multifamily.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="50" customHeight="1">
+      <c r="A30" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>HappyCo</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>https://happy.co/</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>1-888-666-1855</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>Public app/support phone</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>support@happy.co</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>https://happy.co/</t>
-        </is>
-      </c>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>Good maintenance automation fit. Support phone may not route to sales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="44" customHeight="1">
-      <c r="A31" s="4" t="n">
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Sales / multifamily maintenance sales</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Good maintenance automation fit; support phone may route poorly.</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>Who handles new sales for HappyCo maintenance automation?</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>If support-only, find sales email/person later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="50" customHeight="1">
+      <c r="A31" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>eWorkOrders</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>https://eworkorders.com/property-management-maintenance-management-software-cmms/</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>(888) 333-4617</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Official phone</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>https://eworkorders.com/property-management-maintenance-management-software-cmms/</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>Good property maintenance CMMS fit, not fully multifamily-specific.</t>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Sales / property management vertical</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>Property maintenance CMMS, not fully multifamily-specific.</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>Do you want property management maintenance leads in Texas?</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>Good second-wave call.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I31"/>
+  <autoFilter ref="A1:J31"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -1855,80 +2111,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="112" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="118" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Goal</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Call the best public phone number for each vendor and ask who should receive CraneSignal free Texas maintenance-pain sample leads.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Best opener</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Hi, this is Drew with CraneSignal. We are mapping Texas apartment communities showing public maintenance pain signals. I pulled a few accounts your sales team may want. Who is the best person to send that to?</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>What changed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Removed the call-notes PDF template and removed vague named-person instructions. The sheet now gives a best phone number for every company.</t>
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Why website links matter</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Open the website before calling so you can say one sentence that matches their product. Example: for AppWork, mention multifamily maintenance work orders and make-readies.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Best extra caller info</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Ask for, why they might care, first question, confidence, and fallback note are the highest-value fields for a caller.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Number confidence</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>High means official site/help/contact/terms. Medium means public app listing or support line. Low means third-party public listing and should be checked before repeated calls.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>First wave</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Call Tier A first. If a number routes to support, ask for sales, partnerships, business development, or revenue leadership.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Do not say</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Do not say every apartment needs software. Say we found timely accounts with evidence-backed maintenance pain.</t>
         </is>

</xml_diff>

<commit_message>
Reformat CraneSignal call sheet PDF
</commit_message>
<xml_diff>
--- a/docs/call-sheets/cranesignal-maintenance-software-call-sheet-2026-09-21.xlsx
+++ b/docs/call-sheets/cranesignal-maintenance-software-call-sheet-2026-09-21.xlsx
@@ -497,7 +497,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -505,13 +505,13 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -566,7 +566,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="50" customHeight="1">
+    <row r="2" ht="68" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -616,7 +616,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="50" customHeight="1">
+    <row r="3" ht="68" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -666,7 +666,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="50" customHeight="1">
+    <row r="4" ht="68" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -716,7 +716,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="50" customHeight="1">
+    <row r="5" ht="68" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -766,7 +766,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="50" customHeight="1">
+    <row r="6" ht="68" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -816,7 +816,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="50" customHeight="1">
+    <row r="7" ht="68" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -866,7 +866,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="50" customHeight="1">
+    <row r="8" ht="68" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -916,7 +916,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="50" customHeight="1">
+    <row r="9" ht="68" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
@@ -966,7 +966,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="50" customHeight="1">
+    <row r="10" ht="68" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
@@ -1016,7 +1016,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="50" customHeight="1">
+    <row r="11" ht="68" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="50" customHeight="1">
+    <row r="12" ht="68" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
@@ -1116,7 +1116,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="50" customHeight="1">
+    <row r="13" ht="68" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
@@ -1166,7 +1166,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="50" customHeight="1">
+    <row r="14" ht="68" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="50" customHeight="1">
+    <row r="15" ht="68" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
@@ -1266,7 +1266,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="50" customHeight="1">
+    <row r="16" ht="68" customHeight="1">
       <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
@@ -1316,7 +1316,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="50" customHeight="1">
+    <row r="17" ht="68" customHeight="1">
       <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
@@ -1366,7 +1366,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="50" customHeight="1">
+    <row r="18" ht="68" customHeight="1">
       <c r="A18" s="4" t="n">
         <v>17</v>
       </c>
@@ -1416,7 +1416,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="50" customHeight="1">
+    <row r="19" ht="68" customHeight="1">
       <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
@@ -1466,7 +1466,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="50" customHeight="1">
+    <row r="20" ht="68" customHeight="1">
       <c r="A20" s="4" t="n">
         <v>19</v>
       </c>
@@ -1516,7 +1516,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="50" customHeight="1">
+    <row r="21" ht="68" customHeight="1">
       <c r="A21" s="4" t="n">
         <v>20</v>
       </c>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="50" customHeight="1">
+    <row r="22" ht="68" customHeight="1">
       <c r="A22" s="4" t="n">
         <v>21</v>
       </c>
@@ -1616,7 +1616,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="50" customHeight="1">
+    <row r="23" ht="68" customHeight="1">
       <c r="A23" s="4" t="n">
         <v>22</v>
       </c>
@@ -1666,7 +1666,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="50" customHeight="1">
+    <row r="24" ht="68" customHeight="1">
       <c r="A24" s="4" t="n">
         <v>23</v>
       </c>
@@ -1716,7 +1716,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="50" customHeight="1">
+    <row r="25" ht="68" customHeight="1">
       <c r="A25" s="6" t="n">
         <v>24</v>
       </c>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="50" customHeight="1">
+    <row r="26" ht="68" customHeight="1">
       <c r="A26" s="6" t="n">
         <v>25</v>
       </c>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="50" customHeight="1">
+    <row r="27" ht="68" customHeight="1">
       <c r="A27" s="6" t="n">
         <v>26</v>
       </c>
@@ -1866,7 +1866,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="50" customHeight="1">
+    <row r="28" ht="68" customHeight="1">
       <c r="A28" s="6" t="n">
         <v>27</v>
       </c>
@@ -1916,7 +1916,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="50" customHeight="1">
+    <row r="29" ht="68" customHeight="1">
       <c r="A29" s="6" t="n">
         <v>28</v>
       </c>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="50" customHeight="1">
+    <row r="30" ht="68" customHeight="1">
       <c r="A30" s="6" t="n">
         <v>29</v>
       </c>
@@ -2016,7 +2016,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="50" customHeight="1">
+    <row r="31" ht="68" customHeight="1">
       <c r="A31" s="6" t="n">
         <v>30</v>
       </c>
@@ -2101,7 +2101,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2111,7 +2110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2145,24 +2144,24 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Why website links matter</t>
+          <t>PDF format</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Open the website before calling so you can say one sentence that matches their product. Example: for AppWork, mention multifamily maintenance work orders and make-readies.</t>
+          <t>The PDF uses wrapped company cards instead of a dense table so websites, questions, and notes do not get cut off.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Best extra caller info</t>
+          <t>Why website links matter</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Ask for, why they might care, first question, confidence, and fallback note are the highest-value fields for a caller.</t>
+          <t>Open the website before calling so you can say one sentence that matches their product.</t>
         </is>
       </c>
     </row>
@@ -2187,18 +2186,6 @@
       <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Call Tier A first. If a number routes to support, ask for sales, partnerships, business development, or revenue leadership.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Do not say</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Do not say every apartment needs software. Say we found timely accounts with evidence-backed maintenance pain.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add company summaries to CraneSignal call sheet
</commit_message>
<xml_diff>
--- a/docs/call-sheets/cranesignal-maintenance-software-call-sheet-2026-09-21.xlsx
+++ b/docs/call-sheets/cranesignal-maintenance-software-call-sheet-2026-09-21.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Phone Call Sheet'!$A$1:$J$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Phone Call Sheet'!$A$1:$K$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,19 +499,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="38" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -537,36 +538,41 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Best phone</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Ask for</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Why they might care</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>First question</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Fallback / note</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="68" customHeight="1">
+    <row r="2" ht="78" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -587,36 +593,41 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>Multifamily maintenance work orders, inspections, make-readies, and technician workflows.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>+1 347-909-1604</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Sales / founder / revenue leader</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>They sell exactly into multifamily maintenance teams.</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Do you sell into Texas multifamily operators today?</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>If routed to support, ask for sales or partnerships.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="68" customHeight="1">
+    <row r="3" ht="78" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -637,36 +648,41 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Multifamily property operations, maintenance, risk, due diligence, and turn workflows.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>877-995-3662 x513</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Sales / enterprise sales / partnerships</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>They sell property operations and maintenance software to multifamily.</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Would a sourced list of Texas properties with maintenance-risk signals help your sales team?</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Use sales extension first; general extension is x500.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="68" customHeight="1">
+    <row r="4" ht="78" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -687,36 +703,41 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Apartment maintenance CMMS for work orders, preventive maintenance, and reporting.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>888-222-0206 ext. 1</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Sales / account executive</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Clear apartment maintenance/work-order buyer.</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Do you have reps prospecting apartment operators in Texas?</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Use sales option.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="68" customHeight="1">
+    <row r="5" ht="78" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -737,36 +758,41 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>Property inspection software with tenant self-inspections and AI inspection reports.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>+1 530-746-8178</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Medium-high</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Inspection and condition data maps well to move-in and repair pain.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Would properties with inspection or move-in condition complaints be useful leads?</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>If support answers, ask who handles new business.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="68" customHeight="1">
+    <row r="6" ht="78" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -787,36 +813,41 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>AI maintenance coordination, troubleshooting, dispatch, and after-hours support.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>206-900-9466</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Sales / growth / partnerships</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>They handle maintenance coordination, calls, troubleshooting, dispatch.</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Do you want Texas operators showing public unresolved-maintenance pain?</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Ask for the team handling property manager growth.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="68" customHeight="1">
+    <row r="7" ht="78" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -837,36 +868,41 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>Maintenance coordination, vendor network, after-hours response, make-ready, and scheduling.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>913-513-4480</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Maintenance coordination and vendor network fits urgent maintenance pain.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Would a list of Texas operators with visible maintenance backlog signals help?</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Ask for property management sales.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="68" customHeight="1">
+    <row r="8" ht="78" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -887,36 +923,41 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>Work-order and property maintenance management for requests, vendors, assets, and inspections.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>+1 619-752-4422</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Founder / sales / partnerships</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Smaller vendor, clear maintenance workflow fit.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Are you looking for more apartment maintenance software leads in Texas?</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Small company: ask directly for the owner of sales.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="68" customHeight="1">
+    <row r="9" ht="78" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
@@ -937,36 +978,41 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>AI multifamily maintenance and capital operations software.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>+1 647-797-1997</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Sales / partnerships / revenue leader</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>AI multifamily maintenance and capital operations fit.</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Would maintenance-pain evidence help you prioritize Texas accounts?</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>If no sales route, use info@suitespot.ai.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="68" customHeight="1">
+    <row r="10" ht="78" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
@@ -987,36 +1033,41 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>Property maintenance automation for repair coordination and resident/vendor workflows.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>+1 605-646-4102</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Medium-high</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Very strong maintenance automation fit.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Do you want a few Texas properties where residents publicly complain about repairs?</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Phone may route poorly; backup email support@propertymeld.com.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="68" customHeight="1">
+    <row r="11" ht="78" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
@@ -1037,36 +1088,41 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>AI maintenance intake and automation for property operations.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>+1 617-877-8802</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Low-medium</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Founder / sales / Property Meld contact</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>AI maintenance intake fit, but company/contact trail is weaker.</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Who is the right person for AI maintenance sales lead data?</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>If number fails, route through Property Meld because Mezo was acquired.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="68" customHeight="1">
+    <row r="12" ht="78" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
@@ -1087,36 +1143,41 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
+          <t>Building operations platform with maintenance requests, vendor tools, assets, and resident services.</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
           <t>(877) 501-7117</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Sales / multifamily sales</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Building operations and maintenance requests.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>Do you sell into apartment communities where resident operations are visibly strained?</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>US/Canada line.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="68" customHeight="1">
+    <row r="13" ht="78" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
@@ -1137,36 +1198,41 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
+          <t>Resident experience and building operations software for multifamily communities.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
           <t>(844) 800-7109</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Sales / multifamily team</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Resident experience plus building operations.</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>Would maintenance plus resident-experience pain signals help your team?</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Support/general line; ask for Activate Multifamily sales.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="68" customHeight="1">
+    <row r="14" ht="78" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
@@ -1187,36 +1253,41 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
+          <t>Resident app and property hub with payments, maintenance requests, packages, and move-in tools.</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
           <t>+1 773-673-9223</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Medium-high</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Resident app with maintenance requests.</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Do you prospect apartment communities with resident experience issues?</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Backup support@livly.io.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="68" customHeight="1">
+    <row r="15" ht="78" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
@@ -1237,36 +1308,41 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
+          <t>Resident workflow platform for payments, utilities, apps, move-ins, and maintenance requests.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
           <t>1-866-729-5327</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Sales / resident experience sales</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Resident workflow and maintenance request system.</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>Do Texas resident-workflow pain signals help your prospecting?</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Official support line; ask for sales.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="68" customHeight="1">
+    <row r="16" ht="78" customHeight="1">
       <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
@@ -1287,36 +1363,41 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
+          <t>Property inspection and maintenance workflow software with reports and photo documentation.</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
           <t>1 (888) 883-8046</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Inspection and property maintenance workflows.</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>Would inspection/move-in condition complaint leads be useful?</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>Backup contact@snapinspect.com.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="68" customHeight="1">
+    <row r="17" ht="78" customHeight="1">
       <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
@@ -1337,36 +1418,41 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
+          <t>Enterprise building maintenance and property work-order management software.</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
           <t>+1 800 321 8770</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>MRI Angus sales / building maintenance sales</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Enterprise building maintenance and work-order system.</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>Who handles lead data or partnerships for MRI Angus?</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Large company: expect routing.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="68" customHeight="1">
+    <row r="18" ht="78" customHeight="1">
       <c r="A18" s="4" t="n">
         <v>17</v>
       </c>
@@ -1387,36 +1473,41 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
+          <t>Property management platform with maintenance, accounting, leasing, vendor payments, and AI handling.</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
           <t>+1-888-607-3667</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Broad PMS with AI maintenance/work orders.</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>Do you want Texas apartment operators with public maintenance complaints?</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Backup USA number +1-786-373-5842.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="68" customHeight="1">
+    <row r="19" ht="78" customHeight="1">
       <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
@@ -1437,36 +1528,41 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
+          <t>Property management software with resident center, maintenance requests, and maintenance contact center.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
           <t>877-396-7876</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>PMS with maintenance requests and contact center.</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>Who reviews prospecting data partnerships for Buildium sales?</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>RealPage-owned, second wave.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="68" customHeight="1">
+    <row r="20" ht="78" customHeight="1">
       <c r="A20" s="4" t="n">
         <v>19</v>
       </c>
@@ -1487,36 +1583,41 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
+          <t>Multifamily PMS with maintenance, resident portal, contact center, and AI resident assistant.</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
           <t>(888) 702-0971</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Multifamily PMS with maintenance and resident portal.</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>Would Texas operational-pain account lists help ResMan reps?</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>Texas-linked broad PMS.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="68" customHeight="1">
+    <row r="21" ht="78" customHeight="1">
       <c r="A21" s="4" t="n">
         <v>20</v>
       </c>
@@ -1537,36 +1638,41 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
+          <t>Large property management platform with maintenance, resident service, communications, and AI ops.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
           <t>866.648.1536</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>Large PMS with maintenance and resident service.</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>Who handles sales intelligence or lead partnerships?</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Large company; use after sample is strong.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="68" customHeight="1">
+    <row r="22" ht="78" customHeight="1">
       <c r="A22" s="4" t="n">
         <v>21</v>
       </c>
@@ -1587,36 +1693,41 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
+          <t>Property management software for residential, commercial, affordable, HOA, and other portfolios.</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
           <t>(800) 866-1144</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Large PMS serving residential portfolios.</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
         <is>
           <t>Who reviews new account intelligence for Yardi Breeze sales?</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="K22" s="4" t="inlineStr">
         <is>
           <t>Large company; likely hard to route.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="68" customHeight="1">
+    <row r="23" ht="78" customHeight="1">
       <c r="A23" s="4" t="n">
         <v>22</v>
       </c>
@@ -1637,36 +1748,41 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
+          <t>Facilities app for maintenance teams to manage work orders and inspections.</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
           <t>1.800.700.2097</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Facilities product sales / partnerships</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>Facilities app for maintenance work orders and inspections.</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>Would Texas properties with visible maintenance complaints be useful?</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="K23" s="4" t="inlineStr">
         <is>
           <t>Backup sales@entrata.com.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="68" customHeight="1">
+    <row r="24" ht="78" customHeight="1">
       <c r="A24" s="4" t="n">
         <v>23</v>
       </c>
@@ -1687,36 +1803,41 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
+          <t>Smart apartment and property operations tools including tasks, inspections, and resident service.</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
           <t>1 (833) 767-8736</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Sales / SightPlan or operations sales</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Smart operations, resident service, tasks, inspections.</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="J24" s="4" t="inlineStr">
         <is>
           <t>Who handles sales data for property operations products?</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="K24" s="4" t="inlineStr">
         <is>
           <t>Backup help@sightplan.com.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="68" customHeight="1">
+    <row r="25" ht="78" customHeight="1">
       <c r="A25" s="6" t="n">
         <v>24</v>
       </c>
@@ -1737,36 +1858,41 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
+          <t>Enterprise connected CMMS and property operations platform for work orders and vendors.</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
           <t>+91 98848 02586</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>Low-medium</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>Sales / partnerships</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>Enterprise property operations; less apartment-specific.</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="J25" s="6" t="inlineStr">
         <is>
           <t>Do you sell into US multifamily, or mostly commercial facilities?</t>
         </is>
       </c>
-      <c r="J25" s="6" t="inlineStr">
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>Low priority unless they confirm multifamily.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="68" customHeight="1">
+    <row r="26" ht="78" customHeight="1">
       <c r="A26" s="6" t="n">
         <v>25</v>
       </c>
@@ -1787,36 +1913,41 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
+          <t>Facilities and maintenance management software for work orders, PMs, scheduling, and reporting.</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
           <t>+1 (844) 664-4400</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>Sales / property management vertical</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>Facilities and maintenance management.</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
+      <c r="J26" s="6" t="inlineStr">
         <is>
           <t>Do you actively target apartment or property management companies?</t>
         </is>
       </c>
-      <c r="J26" s="6" t="inlineStr">
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>Less apartment-specific.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="68" customHeight="1">
+    <row r="27" ht="78" customHeight="1">
       <c r="A27" s="6" t="n">
         <v>26</v>
       </c>
@@ -1837,36 +1968,41 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
+          <t>Broad CMMS for work orders, preventive maintenance, assets, QR codes, and technicians.</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
           <t>+1 (775) 210-5128</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>Sales / property management use case</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>Broad CMMS, lower apartment specificity.</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
+      <c r="J27" s="6" t="inlineStr">
         <is>
           <t>Do you have a multifamily/property management vertical?</t>
         </is>
       </c>
-      <c r="J27" s="6" t="inlineStr">
+      <c r="K27" s="6" t="inlineStr">
         <is>
           <t>Only pursue if they say yes.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="68" customHeight="1">
+    <row r="28" ht="78" customHeight="1">
       <c r="A28" s="6" t="n">
         <v>27</v>
       </c>
@@ -1887,36 +2023,41 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
+          <t>CMMS/work-order platform with property management and maintenance operations use cases.</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
           <t>+1 (323) 880-0280</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>Sales / property management use case</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>Broad CMMS with property management use case.</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr">
+      <c r="J28" s="6" t="inlineStr">
         <is>
           <t>Do you have a team selling into multifamily or apartment operators?</t>
         </is>
       </c>
-      <c r="J28" s="6" t="inlineStr">
+      <c r="K28" s="6" t="inlineStr">
         <is>
           <t>Lower priority than apartment-native vendors.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="68" customHeight="1">
+    <row r="29" ht="78" customHeight="1">
       <c r="A29" s="6" t="n">
         <v>28</v>
       </c>
@@ -1937,36 +2078,41 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
+          <t>Maintenance operations and work-order software for teams and facilities.</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
           <t>415-548-4001</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>Sales / property management use case</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="I29" s="6" t="inlineStr">
         <is>
           <t>Broad maintenance ops software.</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr">
+      <c r="J29" s="6" t="inlineStr">
         <is>
           <t>Do you sell into apartment maintenance teams or mostly industrial?</t>
         </is>
       </c>
-      <c r="J29" s="6" t="inlineStr">
+      <c r="K29" s="6" t="inlineStr">
         <is>
           <t>Lower priority unless they confirm multifamily.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="68" customHeight="1">
+    <row r="30" ht="78" customHeight="1">
       <c r="A30" s="6" t="n">
         <v>29</v>
       </c>
@@ -1987,36 +2133,41 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
+          <t>Property operations software with AI maintenance automation, work orders, and inspections.</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
           <t>1-888-666-1855</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Sales / multifamily maintenance sales</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
         <is>
           <t>Good maintenance automation fit; support phone may route poorly.</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr">
+      <c r="J30" s="6" t="inlineStr">
         <is>
           <t>Who handles new sales for HappyCo maintenance automation?</t>
         </is>
       </c>
-      <c r="J30" s="6" t="inlineStr">
+      <c r="K30" s="6" t="inlineStr">
         <is>
           <t>If support-only, find sales email/person later.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="68" customHeight="1">
+    <row r="31" ht="78" customHeight="1">
       <c r="A31" s="6" t="n">
         <v>30</v>
       </c>
@@ -2037,37 +2188,42 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
+          <t>Property maintenance CMMS for work orders, assets, vendors, inspections, and compliance.</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
           <t>(888) 333-4617</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Sales / property management vertical</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
         <is>
           <t>Property maintenance CMMS, not fully multifamily-specific.</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="J31" s="6" t="inlineStr">
         <is>
           <t>Do you want property management maintenance leads in Texas?</t>
         </is>
       </c>
-      <c r="J31" s="6" t="inlineStr">
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>Good second-wave call.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J31"/>
+  <autoFilter ref="A1:K31"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -2110,7 +2266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2144,48 +2300,24 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>PDF format</t>
+          <t>Summary column</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>The PDF uses wrapped company cards instead of a dense table so websites, questions, and notes do not get cut off.</t>
+          <t>Use this to quickly understand what the company does before dialing.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Why website links matter</t>
+          <t>Number confidence</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Open the website before calling so you can say one sentence that matches their product.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Number confidence</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
           <t>High means official site/help/contact/terms. Medium means public app listing or support line. Low means third-party public listing and should be checked before repeated calls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>First wave</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Call Tier A first. If a number routes to support, ask for sales, partnerships, business development, or revenue leadership.</t>
         </is>
       </c>
     </row>

</xml_diff>